<commit_message>
Add V4.8 version of PTH design
Include the new resistor for target speed selection.
</commit_message>
<xml_diff>
--- a/AstroEQ-Hardware/SMD/AstroEQ V4.8 BOM.xlsx
+++ b/AstroEQ-Hardware/SMD/AstroEQ V4.8 BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Thomas\Documents\GitHub\AstroEQ\AstroEQ-Hardware\SMD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B943192-1FE0-47E4-831E-04DCE94BBD84}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{307F465B-F86C-4AB6-B2BE-B5A720FED433}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="47820" windowHeight="19965" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1812,7 +1812,7 @@
         <v>110</v>
       </c>
       <c r="D19" s="8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>201</v>

</xml_diff>